<commit_message>
update to match naming convention and fix .env.example key name
</commit_message>
<xml_diff>
--- a/OPEN_AI_API/03_RESULTS/01_AI_RESPONSE.xlsx
+++ b/OPEN_AI_API/03_RESULTS/01_AI_RESPONSE.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\300FMASTERCLASS\03_PYTHON_MC202602\10_PYTHON_MEETING_10\OPEN_AI_API\03_RESULTS\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F3D820-69A2-48EF-B7DA-48BE38EA0079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
   <si>
     <t>dashboard_id</t>
   </si>
@@ -55,87 +49,84 @@
     <t>Chart 1/ Comparison between purchase order, goods receipt, invoice, payment value per month</t>
   </si>
   <si>
-    <t>Invoice Excess over Purchase</t>
+    <t>High PO vs. Invoice Discrepancy</t>
   </si>
   <si>
     <t>High</t>
   </si>
   <si>
-    <t>Invoices exceed Purchase Orders in multiple months</t>
-  </si>
-  <si>
-    <t>Potential for inflated costs and tax evasion</t>
-  </si>
-  <si>
-    <t>Audit purchasing budgets and review invoices thoroughly.</t>
-  </si>
-  <si>
-    <t>The analysis of the comparison between purchase orders, goods receipts, invoices, and payments has revealed significant discrepancies that warrant attention. 
-- There are multiple instances where Invoice values exceed Purchase Order values, suggesting possible over-estimation of purchasing budgets and the risk of fictitious invoicing.
-- Payments do not consistently match the level of invoicing, indicating that some invoices may lack legitimacy.
-- These discrepancies in Goods Receipts being lower than expected compared to Invoice values highlight potential issues in inventory management, suggesting goods could be unrecorded or intercepted.
-To mitigate these risks, it is recommended to perform comprehensive audits on purchasing processes, tighten controls over invoices and payments, and ensure that inventory handling aligns with goods receipts. These actions will not only enhance financial accuracy but will also reinforce the overall integrity of the procurement cycle in SAP.</t>
-  </si>
-  <si>
-    <t>Invoice Exceeds Payment</t>
+    <t>PO values are significantly lower than invoices.</t>
+  </si>
+  <si>
+    <t>Possible budget overestimation or control failure.</t>
+  </si>
+  <si>
+    <t>Conduct an audit to reconcile purchase orders and invoices.</t>
+  </si>
+  <si>
+    <t>The analysis of Purchase Orders, Goods Receipts, Invoices, and Payments shows notable discrepancies and patterns. The evaluation highlighted significant issues, including higher invoice values compared to payments and consistently lower goods receipt values than invoices. These trends raise concerns about potential fictitious invoices and ineffective inventory management, which could lead to financial losses and compliance risks.
+Immediate attention is required to address the high discrepancies in Purchase Orders versus Invoices, as this could indicate planning or approval process failures. Furthermore, the lower values of Goods Receipts in relation to Invoices necessitate a closer investigation into potential inventory management issues. Implementing rigorous audits, reviewing process controls, and ensuring proper documentation will enhance efficiency and mitigate risks across the Order to Cash process.</t>
+  </si>
+  <si>
+    <t>Lower GR compared to Invoice</t>
   </si>
   <si>
     <t>Medium</t>
   </si>
   <si>
-    <t>Several months show invoices &gt; payments</t>
-  </si>
-  <si>
-    <t>Risk of fictitious invoices</t>
-  </si>
-  <si>
-    <t>Implement tighter controls on invoice approval process.</t>
-  </si>
-  <si>
-    <t>Low Goods Receipt</t>
-  </si>
-  <si>
-    <t>Goods Receipts consistently lower than Invoices</t>
-  </si>
-  <si>
-    <t>Risk of inventory theft or mismanagement</t>
-  </si>
-  <si>
-    <t>Conduct inventory audits and review receipt logging.</t>
-  </si>
-  <si>
-    <t>Purchase Order Low vs Invoice</t>
-  </si>
-  <si>
-    <t>January and March show Purchase Orders &lt; Invoices</t>
-  </si>
-  <si>
-    <t>Purchasing process not properly followed</t>
-  </si>
-  <si>
-    <t>Encourage adherence to SAP materials management module.</t>
-  </si>
-  <si>
-    <t>Goods Receipt Approaching Orders</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Some months show Goods Receipts close to POs</t>
-  </si>
-  <si>
-    <t>Indicator of potential supplier over-delivery</t>
-  </si>
-  <si>
-    <t>Review supplier delivery metrics and maintain strict approvals.</t>
+    <t>GR values are lower than Invoice values consistently.</t>
+  </si>
+  <si>
+    <t>Risk of inventory mismanagement or supplier fraud.</t>
+  </si>
+  <si>
+    <t>Review Goods Receipt processes and compliance thoroughly.</t>
+  </si>
+  <si>
+    <t>Invoice higher than Payment</t>
+  </si>
+  <si>
+    <t>Invoices exceeding payment values in multiple months.</t>
+  </si>
+  <si>
+    <t>Risk of fictitious billing and financial manipulation.</t>
+  </si>
+  <si>
+    <t>Perform a detailed invoice validation audit to check authenticity.</t>
+  </si>
+  <si>
+    <t>Low PO values relative to GR</t>
+  </si>
+  <si>
+    <t>PO amounts are considerably lower than corresponding GRs.</t>
+  </si>
+  <si>
+    <t>Risk of irregular procurement practices.</t>
+  </si>
+  <si>
+    <t>Investigate procurement processes and ensure approvals are enforced.</t>
+  </si>
+  <si>
+    <t>Consistent patterns of disparity</t>
+  </si>
+  <si>
+    <t>Persistent inconsistencies across months.</t>
+  </si>
+  <si>
+    <t>Suggests systemic inefficiencies in workflows.</t>
+  </si>
+  <si>
+    <t>Recommend comprehensive process review and efficiency improvements.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0;[Red]-#,##0"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,52 +160,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="38" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf/>
     <dxf>
-      <numFmt numFmtId="6" formatCode="#,##0;[Red]\-#,##0"/>
+      <numFmt numFmtId="164" formatCode="#,##0;[Red]-#,##0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Frame0" displayName="Frame0" ref="A1:I6" totalsRowShown="0">
-  <autoFilter ref="A1:I6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:I6" totalsRowShown="0">
+  <autoFilter ref="A1:I6"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="dashboard_id"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="task_index" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="chart_title"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Issue"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Priority"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Observation"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Risk"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Recommendation"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Executive Summary"/>
+    <tableColumn id="1" name="dashboard_id" dataDxfId="0"/>
+    <tableColumn id="2" name="task_index" dataDxfId="1"/>
+    <tableColumn id="3" name="chart_title" dataDxfId="0"/>
+    <tableColumn id="4" name="Issue" dataDxfId="0"/>
+    <tableColumn id="5" name="Priority" dataDxfId="0"/>
+    <tableColumn id="6" name="Observation" dataDxfId="0"/>
+    <tableColumn id="7" name="Risk" dataDxfId="0"/>
+    <tableColumn id="8" name="Recommendation" dataDxfId="0"/>
+    <tableColumn id="9" name="Executive Summary" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -252,7 +236,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -286,7 +270,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -321,10 +304,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -497,11 +479,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -530,7 +512,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
@@ -559,7 +541,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -588,7 +570,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -617,7 +599,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -646,7 +628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -660,16 +642,16 @@
         <v>30</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>16</v>
@@ -677,9 +659,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>